<commit_message>
Update GP by Buyer - assign 76HPSB MPNs (Jake/Stephanie)
All 2024 lines now assigned

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -438,10 +438,10 @@
         <v>Jake Harris</v>
       </c>
       <c r="B2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C2">
-        <v>4988.09</v>
+        <v>4996.77</v>
       </c>
       <c r="D2" t="str">
         <v>38.0%</v>
@@ -453,7 +453,7 @@
         <v>27.5%</v>
       </c>
       <c r="G2">
-        <v>3983.73</v>
+        <v>3992.41</v>
       </c>
       <c r="H2" t="str">
         <v>39.8%</v>
@@ -502,13 +502,13 @@
         <v>Stephanie Hill</v>
       </c>
       <c r="B4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4">
-        <v>145.75</v>
+        <v>161.41</v>
       </c>
       <c r="D4" t="str">
-        <v>32.0%</v>
+        <v>31.6%</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -517,10 +517,10 @@
         <v/>
       </c>
       <c r="G4">
-        <v>145.39</v>
+        <v>161.05</v>
       </c>
       <c r="H4" t="str">
-        <v>32.0%</v>
+        <v>31.6%</v>
       </c>
       <c r="I4">
         <v>0.36</v>
@@ -595,71 +595,39 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Unmatched</v>
+        <v>TOTAL</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>130</v>
       </c>
       <c r="C7">
-        <v>24.34</v>
+        <v>8151.03</v>
       </c>
       <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
+        <v>33.3%</v>
+      </c>
+      <c r="E7">
+        <v>2758.02</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>23.7%</v>
       </c>
       <c r="G7">
-        <v>24.34</v>
+        <v>4760.47</v>
       </c>
       <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
+        <v>36.1%</v>
+      </c>
+      <c r="I7">
+        <v>632.54</v>
       </c>
       <c r="J7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B8">
-        <v>130</v>
-      </c>
-      <c r="C8">
-        <v>8151.03</v>
-      </c>
-      <c r="D8" t="str">
-        <v>33.3%</v>
-      </c>
-      <c r="E8">
-        <v>2758.02</v>
-      </c>
-      <c r="F8" t="str">
-        <v>23.7%</v>
-      </c>
-      <c r="G8">
-        <v>4760.47</v>
-      </c>
-      <c r="H8" t="str">
-        <v>36.1%</v>
-      </c>
-      <c r="I8">
-        <v>632.54</v>
-      </c>
-      <c r="J8" t="str">
         <v>40.1%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -901,7 +869,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -931,10 +899,10 @@
         <v>Jake Harris</v>
       </c>
       <c r="B2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C2">
-        <v>4988.09</v>
+        <v>4996.77</v>
       </c>
       <c r="D2">
         <v>240</v>
@@ -943,10 +911,10 @@
         <v>7399.05</v>
       </c>
       <c r="F2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G2">
-        <v>12387.14</v>
+        <v>12395.82</v>
       </c>
     </row>
     <row r="3">
@@ -1000,10 +968,10 @@
         <v>Stephanie Hill</v>
       </c>
       <c r="B5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5">
-        <v>145.75</v>
+        <v>161.41</v>
       </c>
       <c r="D5">
         <v>109</v>
@@ -1012,10 +980,10 @@
         <v>1308.11</v>
       </c>
       <c r="F5">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G5">
-        <v>1453.86</v>
+        <v>1469.52</v>
       </c>
     </row>
     <row r="6">
@@ -1043,53 +1011,30 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Unmatched 2024</v>
+        <v>TOTAL</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>130</v>
       </c>
       <c r="C7">
-        <v>24.34</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
+        <v>8151.03</v>
+      </c>
+      <c r="D7">
+        <v>469</v>
+      </c>
+      <c r="E7">
+        <v>16830.95</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>599</v>
       </c>
       <c r="G7">
-        <v>24.34</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B8">
-        <v>130</v>
-      </c>
-      <c r="C8">
-        <v>8151.03</v>
-      </c>
-      <c r="D8">
-        <v>469</v>
-      </c>
-      <c r="E8">
-        <v>16830.95</v>
-      </c>
-      <c r="F8">
-        <v>599</v>
-      </c>
-      <c r="G8">
         <v>24981.98</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Cumulative tab with buyer/customer breakdown
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
@@ -869,29 +869,38 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:J7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Buyer</v>
       </c>
       <c r="B1" t="str">
-        <v>2024 Lines</v>
+        <v>Total Lines</v>
       </c>
       <c r="C1" t="str">
-        <v>2024 GP</v>
+        <v>Total GP</v>
       </c>
       <c r="D1" t="str">
-        <v>2025 Lines</v>
+        <v>Total Margin</v>
       </c>
       <c r="E1" t="str">
-        <v>2025 GP</v>
+        <v>VM Services GP</v>
       </c>
       <c r="F1" t="str">
-        <v>Total Lines</v>
+        <v>VM Services Margin</v>
       </c>
       <c r="G1" t="str">
-        <v>Total GP</v>
+        <v>Naprotek GP</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Naprotek Margin</v>
+      </c>
+      <c r="I1" t="str">
+        <v>LAM Plexus GP</v>
+      </c>
+      <c r="J1" t="str">
+        <v>LAM Plexus Margin</v>
       </c>
     </row>
     <row r="2">
@@ -899,22 +908,31 @@
         <v>Jake Harris</v>
       </c>
       <c r="B2">
-        <v>65</v>
+        <v>305</v>
       </c>
       <c r="C2">
-        <v>4996.77</v>
-      </c>
-      <c r="D2">
-        <v>240</v>
+        <v>12395.82</v>
+      </c>
+      <c r="D2" t="str">
+        <v>38.3%</v>
       </c>
       <c r="E2">
-        <v>7399.05</v>
-      </c>
-      <c r="F2">
-        <v>305</v>
+        <v>1759.24</v>
+      </c>
+      <c r="F2" t="str">
+        <v>46.8%</v>
       </c>
       <c r="G2">
-        <v>12395.82</v>
+        <v>9858.89</v>
+      </c>
+      <c r="H2" t="str">
+        <v>37.6%</v>
+      </c>
+      <c r="I2">
+        <v>777.69</v>
+      </c>
+      <c r="J2" t="str">
+        <v>30.8%</v>
       </c>
     </row>
     <row r="3">
@@ -922,22 +940,31 @@
         <v>Tracy Xie</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="C3">
-        <v>97.98</v>
-      </c>
-      <c r="D3">
-        <v>40</v>
+        <v>6962.59</v>
+      </c>
+      <c r="D3" t="str">
+        <v>50.6%</v>
       </c>
       <c r="E3">
-        <v>6864.61</v>
-      </c>
-      <c r="F3">
-        <v>46</v>
+        <v>70.35</v>
+      </c>
+      <c r="F3" t="str">
+        <v>49.9%</v>
       </c>
       <c r="G3">
-        <v>6962.59</v>
+        <v>6707.82</v>
+      </c>
+      <c r="H3" t="str">
+        <v>52.3%</v>
+      </c>
+      <c r="I3">
+        <v>184.42</v>
+      </c>
+      <c r="J3" t="str">
+        <v>24.6%</v>
       </c>
     </row>
     <row r="4">
@@ -945,22 +972,31 @@
         <v>Edgar Santana</v>
       </c>
       <c r="B4">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="C4">
-        <v>2769</v>
-      </c>
-      <c r="D4">
-        <v>52</v>
+        <v>3641.94</v>
+      </c>
+      <c r="D4" t="str">
+        <v>25.7%</v>
       </c>
       <c r="E4">
-        <v>872.94</v>
-      </c>
-      <c r="F4">
-        <v>75</v>
+        <v>2461.71</v>
+      </c>
+      <c r="F4" t="str">
+        <v>23.5%</v>
       </c>
       <c r="G4">
-        <v>3641.94</v>
+        <v>893.6</v>
+      </c>
+      <c r="H4" t="str">
+        <v>25.8%</v>
+      </c>
+      <c r="I4">
+        <v>286.63</v>
+      </c>
+      <c r="J4" t="str">
+        <v>40.3%</v>
       </c>
     </row>
     <row r="5">
@@ -968,22 +1004,31 @@
         <v>Stephanie Hill</v>
       </c>
       <c r="B5">
-        <v>23</v>
+        <v>132</v>
       </c>
       <c r="C5">
-        <v>161.41</v>
-      </c>
-      <c r="D5">
-        <v>109</v>
+        <v>1469.52</v>
+      </c>
+      <c r="D5" t="str">
+        <v>33.6%</v>
       </c>
       <c r="E5">
-        <v>1308.11</v>
-      </c>
-      <c r="F5">
-        <v>132</v>
+        <v>378.37</v>
+      </c>
+      <c r="F5" t="str">
+        <v>38.1%</v>
       </c>
       <c r="G5">
-        <v>1469.52</v>
+        <v>1075.28</v>
+      </c>
+      <c r="H5" t="str">
+        <v>32.1%</v>
+      </c>
+      <c r="I5">
+        <v>15.87</v>
+      </c>
+      <c r="J5" t="str">
+        <v>26.6%</v>
       </c>
     </row>
     <row r="6">
@@ -991,22 +1036,31 @@
         <v>Daniel</v>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="C6">
-        <v>125.87</v>
-      </c>
-      <c r="D6">
-        <v>28</v>
+        <v>512.1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>20.3%</v>
       </c>
       <c r="E6">
-        <v>386.23</v>
-      </c>
-      <c r="F6">
-        <v>41</v>
+        <v>203.87</v>
+      </c>
+      <c r="F6" t="str">
+        <v>25.2%</v>
       </c>
       <c r="G6">
-        <v>512.1</v>
+        <v>244.64</v>
+      </c>
+      <c r="H6" t="str">
+        <v>15.5%</v>
+      </c>
+      <c r="I6">
+        <v>63.6</v>
+      </c>
+      <c r="J6" t="str">
+        <v>34.0%</v>
       </c>
     </row>
     <row r="7">
@@ -1014,27 +1068,36 @@
         <v>TOTAL</v>
       </c>
       <c r="B7">
-        <v>130</v>
+        <v>599</v>
       </c>
       <c r="C7">
-        <v>8151.03</v>
-      </c>
-      <c r="D7">
-        <v>469</v>
+        <v>24981.98</v>
+      </c>
+      <c r="D7" t="str">
+        <v>37.5%</v>
       </c>
       <c r="E7">
-        <v>16830.95</v>
-      </c>
-      <c r="F7">
-        <v>599</v>
+        <v>4873.54</v>
+      </c>
+      <c r="F7" t="str">
+        <v>29.9%</v>
       </c>
       <c r="G7">
-        <v>24981.98</v>
+        <v>18780.23</v>
+      </c>
+      <c r="H7" t="str">
+        <v>39.6%</v>
+      </c>
+      <c r="I7">
+        <v>1328.21</v>
+      </c>
+      <c r="J7" t="str">
+        <v>32.5%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify GP by Buyer - total lines/margin, GP by customer
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,19 +418,10 @@
         <v>VM Services GP</v>
       </c>
       <c r="F1" t="str">
-        <v>VM Services Margin</v>
+        <v>Naprotek GP</v>
       </c>
       <c r="G1" t="str">
-        <v>Naprotek GP</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Naprotek Margin</v>
-      </c>
-      <c r="I1" t="str">
         <v>LAM Plexus GP</v>
-      </c>
-      <c r="J1" t="str">
-        <v>LAM Plexus Margin</v>
       </c>
     </row>
     <row r="2">
@@ -449,20 +440,11 @@
       <c r="E2">
         <v>449.38</v>
       </c>
-      <c r="F2" t="str">
-        <v>27.5%</v>
+      <c r="F2">
+        <v>3992.41</v>
       </c>
       <c r="G2">
-        <v>3992.41</v>
-      </c>
-      <c r="H2" t="str">
-        <v>39.8%</v>
-      </c>
-      <c r="I2">
         <v>554.98</v>
-      </c>
-      <c r="J2" t="str">
-        <v>36.6%</v>
       </c>
     </row>
     <row r="3">
@@ -481,20 +463,11 @@
       <c r="E3">
         <v>2291.62</v>
       </c>
-      <c r="F3" t="str">
-        <v>22.9%</v>
+      <c r="F3">
+        <v>400.18</v>
       </c>
       <c r="G3">
-        <v>400.18</v>
-      </c>
-      <c r="H3" t="str">
-        <v>28.1%</v>
-      </c>
-      <c r="I3">
         <v>77.2</v>
-      </c>
-      <c r="J3" t="str">
-        <v>59.5%</v>
       </c>
     </row>
     <row r="4">
@@ -513,20 +486,11 @@
       <c r="E4" t="str">
         <v/>
       </c>
-      <c r="F4" t="str">
-        <v/>
+      <c r="F4">
+        <v>161.05</v>
       </c>
       <c r="G4">
-        <v>161.05</v>
-      </c>
-      <c r="H4" t="str">
-        <v>31.6%</v>
-      </c>
-      <c r="I4">
         <v>0.36</v>
-      </c>
-      <c r="J4" t="str">
-        <v>24.1%</v>
       </c>
     </row>
     <row r="5">
@@ -545,19 +509,10 @@
       <c r="E5">
         <v>17.02</v>
       </c>
-      <c r="F5" t="str">
-        <v>16.8%</v>
-      </c>
-      <c r="G5">
+      <c r="F5">
         <v>108.85</v>
       </c>
-      <c r="H5" t="str">
-        <v>43.2%</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
+      <c r="G5" t="str">
         <v/>
       </c>
     </row>
@@ -577,19 +532,10 @@
       <c r="E6" t="str">
         <v/>
       </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6">
+      <c r="F6">
         <v>97.98</v>
       </c>
-      <c r="H6" t="str">
-        <v>8.5%</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
+      <c r="G6" t="str">
         <v/>
       </c>
     </row>
@@ -609,32 +555,23 @@
       <c r="E7">
         <v>2758.02</v>
       </c>
-      <c r="F7" t="str">
-        <v>23.7%</v>
+      <c r="F7">
+        <v>4760.47</v>
       </c>
       <c r="G7">
-        <v>4760.47</v>
-      </c>
-      <c r="H7" t="str">
-        <v>36.1%</v>
-      </c>
-      <c r="I7">
         <v>632.54</v>
-      </c>
-      <c r="J7" t="str">
-        <v>40.1%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -653,19 +590,10 @@
         <v>VM Services GP</v>
       </c>
       <c r="F1" t="str">
-        <v>VM Services Margin</v>
+        <v>Naprotek GP</v>
       </c>
       <c r="G1" t="str">
-        <v>Naprotek GP</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Naprotek Margin</v>
-      </c>
-      <c r="I1" t="str">
         <v>LAM Plexus GP</v>
-      </c>
-      <c r="J1" t="str">
-        <v>LAM Plexus Margin</v>
       </c>
     </row>
     <row r="2">
@@ -684,20 +612,11 @@
       <c r="E2">
         <v>1309.86</v>
       </c>
-      <c r="F2" t="str">
-        <v>51.5%</v>
+      <c r="F2">
+        <v>5866.48</v>
       </c>
       <c r="G2">
-        <v>5866.48</v>
-      </c>
-      <c r="H2" t="str">
-        <v>36.9%</v>
-      </c>
-      <c r="I2">
         <v>222.71</v>
-      </c>
-      <c r="J2" t="str">
-        <v>27.9%</v>
       </c>
     </row>
     <row r="3">
@@ -716,20 +635,11 @@
       <c r="E3">
         <v>70.35</v>
       </c>
-      <c r="F3" t="str">
-        <v>49.9%</v>
+      <c r="F3">
+        <v>6609.84</v>
       </c>
       <c r="G3">
-        <v>6609.84</v>
-      </c>
-      <c r="H3" t="str">
-        <v>52.9%</v>
-      </c>
-      <c r="I3">
         <v>184.42</v>
-      </c>
-      <c r="J3" t="str">
-        <v>24.6%</v>
       </c>
     </row>
     <row r="4">
@@ -748,20 +658,11 @@
       <c r="E4">
         <v>378.37</v>
       </c>
-      <c r="F4" t="str">
-        <v>38.1%</v>
+      <c r="F4">
+        <v>914.23</v>
       </c>
       <c r="G4">
-        <v>914.23</v>
-      </c>
-      <c r="H4" t="str">
-        <v>32.3%</v>
-      </c>
-      <c r="I4">
         <v>15.51</v>
-      </c>
-      <c r="J4" t="str">
-        <v>27.0%</v>
       </c>
     </row>
     <row r="5">
@@ -780,20 +681,11 @@
       <c r="E5">
         <v>170.09</v>
       </c>
-      <c r="F5" t="str">
-        <v>44.3%</v>
+      <c r="F5">
+        <v>493.42</v>
       </c>
       <c r="G5">
-        <v>493.42</v>
-      </c>
-      <c r="H5" t="str">
-        <v>24.7%</v>
-      </c>
-      <c r="I5">
         <v>209.43</v>
-      </c>
-      <c r="J5" t="str">
-        <v>32.1%</v>
       </c>
     </row>
     <row r="6">
@@ -812,20 +704,11 @@
       <c r="E6">
         <v>186.85</v>
       </c>
-      <c r="F6" t="str">
-        <v>28.7%</v>
+      <c r="F6">
+        <v>135.79</v>
       </c>
       <c r="G6">
-        <v>135.79</v>
-      </c>
-      <c r="H6" t="str">
-        <v>7.4%</v>
-      </c>
-      <c r="I6">
         <v>63.6</v>
-      </c>
-      <c r="J6" t="str">
-        <v>34.0%</v>
       </c>
     </row>
     <row r="7">
@@ -844,32 +727,23 @@
       <c r="E7">
         <v>2115.52</v>
       </c>
-      <c r="F7" t="str">
-        <v>44.9%</v>
+      <c r="F7">
+        <v>14019.76</v>
       </c>
       <c r="G7">
-        <v>14019.76</v>
-      </c>
-      <c r="H7" t="str">
-        <v>41.0%</v>
-      </c>
-      <c r="I7">
         <v>695.67</v>
-      </c>
-      <c r="J7" t="str">
-        <v>28.5%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -888,19 +762,10 @@
         <v>VM Services GP</v>
       </c>
       <c r="F1" t="str">
-        <v>VM Services Margin</v>
+        <v>Naprotek GP</v>
       </c>
       <c r="G1" t="str">
-        <v>Naprotek GP</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Naprotek Margin</v>
-      </c>
-      <c r="I1" t="str">
         <v>LAM Plexus GP</v>
-      </c>
-      <c r="J1" t="str">
-        <v>LAM Plexus Margin</v>
       </c>
     </row>
     <row r="2">
@@ -919,20 +784,11 @@
       <c r="E2">
         <v>1759.24</v>
       </c>
-      <c r="F2" t="str">
-        <v>46.8%</v>
+      <c r="F2">
+        <v>9858.89</v>
       </c>
       <c r="G2">
-        <v>9858.89</v>
-      </c>
-      <c r="H2" t="str">
-        <v>37.6%</v>
-      </c>
-      <c r="I2">
         <v>777.69</v>
-      </c>
-      <c r="J2" t="str">
-        <v>30.8%</v>
       </c>
     </row>
     <row r="3">
@@ -951,20 +807,11 @@
       <c r="E3">
         <v>70.35</v>
       </c>
-      <c r="F3" t="str">
-        <v>49.9%</v>
+      <c r="F3">
+        <v>6707.82</v>
       </c>
       <c r="G3">
-        <v>6707.82</v>
-      </c>
-      <c r="H3" t="str">
-        <v>52.3%</v>
-      </c>
-      <c r="I3">
         <v>184.42</v>
-      </c>
-      <c r="J3" t="str">
-        <v>24.6%</v>
       </c>
     </row>
     <row r="4">
@@ -983,20 +830,11 @@
       <c r="E4">
         <v>2461.71</v>
       </c>
-      <c r="F4" t="str">
-        <v>23.5%</v>
+      <c r="F4">
+        <v>893.6</v>
       </c>
       <c r="G4">
-        <v>893.6</v>
-      </c>
-      <c r="H4" t="str">
-        <v>25.8%</v>
-      </c>
-      <c r="I4">
         <v>286.63</v>
-      </c>
-      <c r="J4" t="str">
-        <v>40.3%</v>
       </c>
     </row>
     <row r="5">
@@ -1015,20 +853,11 @@
       <c r="E5">
         <v>378.37</v>
       </c>
-      <c r="F5" t="str">
-        <v>38.1%</v>
+      <c r="F5">
+        <v>1075.28</v>
       </c>
       <c r="G5">
-        <v>1075.28</v>
-      </c>
-      <c r="H5" t="str">
-        <v>32.1%</v>
-      </c>
-      <c r="I5">
         <v>15.87</v>
-      </c>
-      <c r="J5" t="str">
-        <v>26.6%</v>
       </c>
     </row>
     <row r="6">
@@ -1047,20 +876,11 @@
       <c r="E6">
         <v>203.87</v>
       </c>
-      <c r="F6" t="str">
-        <v>25.2%</v>
+      <c r="F6">
+        <v>244.64</v>
       </c>
       <c r="G6">
-        <v>244.64</v>
-      </c>
-      <c r="H6" t="str">
-        <v>15.5%</v>
-      </c>
-      <c r="I6">
         <v>63.6</v>
-      </c>
-      <c r="J6" t="str">
-        <v>34.0%</v>
       </c>
     </row>
     <row r="7">
@@ -1079,25 +899,16 @@
       <c r="E7">
         <v>4873.54</v>
       </c>
-      <c r="F7" t="str">
-        <v>29.9%</v>
+      <c r="F7">
+        <v>18780.23</v>
       </c>
       <c r="G7">
-        <v>18780.23</v>
-      </c>
-      <c r="H7" t="str">
-        <v>39.6%</v>
-      </c>
-      <c r="I7">
         <v>1328.21</v>
-      </c>
-      <c r="J7" t="str">
-        <v>32.5%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Merge Daniel into Edgar on Cumulative tab
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/GP_by_Buyer_Final.xlsx
@@ -743,7 +743,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -819,22 +819,22 @@
         <v>Edgar Santana</v>
       </c>
       <c r="B4">
-        <v>75</v>
+        <v>116</v>
       </c>
       <c r="C4">
-        <v>3641.94</v>
+        <v>4154.04</v>
       </c>
       <c r="D4" t="str">
-        <v>25.7%</v>
+        <v>24.9%</v>
       </c>
       <c r="E4">
-        <v>2461.71</v>
+        <v>2665.58</v>
       </c>
       <c r="F4">
-        <v>893.6</v>
+        <v>1138.24</v>
       </c>
       <c r="G4">
-        <v>286.63</v>
+        <v>350.23</v>
       </c>
     </row>
     <row r="5">
@@ -862,53 +862,30 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Daniel</v>
+        <v>TOTAL</v>
       </c>
       <c r="B6">
-        <v>41</v>
+        <v>599</v>
       </c>
       <c r="C6">
-        <v>512.1</v>
+        <v>24981.98</v>
       </c>
       <c r="D6" t="str">
-        <v>20.3%</v>
+        <v>37.5%</v>
       </c>
       <c r="E6">
-        <v>203.87</v>
+        <v>4873.54</v>
       </c>
       <c r="F6">
-        <v>244.64</v>
+        <v>18780.23</v>
       </c>
       <c r="G6">
-        <v>63.6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B7">
-        <v>599</v>
-      </c>
-      <c r="C7">
-        <v>24981.98</v>
-      </c>
-      <c r="D7" t="str">
-        <v>37.5%</v>
-      </c>
-      <c r="E7">
-        <v>4873.54</v>
-      </c>
-      <c r="F7">
-        <v>18780.23</v>
-      </c>
-      <c r="G7">
         <v>1328.21</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>